<commit_message>
Way too much catchup
</commit_message>
<xml_diff>
--- a/data/All_Sites_Calculated (with z star).xlsx
+++ b/data/All_Sites_Calculated (with z star).xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,13 +10,26 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="21" documentId="8_{4274A576-6E2E-4B05-A1BB-A686EE3EC67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9A7CE96-C753-42A1-BF50-4526C44F1DDC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A73E911E-D0AA-46A2-B8CD-3070576D2DAB}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{A73E911E-D0AA-46A2-B8CD-3070576D2DAB}"/>
   </bookViews>
   <sheets>
     <sheet name="All_Sites_Calculated (with z st" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -2588,6 +2601,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>